<commit_message>
Same small changes (not losing them this time)
</commit_message>
<xml_diff>
--- a/backend/fuel-market-information/fuel-market-information-template.xlsx
+++ b/backend/fuel-market-information/fuel-market-information-template.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/NICCP-AI/backend/fuel-market-information/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:3_{297C9F4D-5BEC-4077-8986-513ACDF59508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{775EC94A-13D7-4A0E-B9CA-FB7C5F7AFCEB}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:3_{297C9F4D-5BEC-4077-8986-513ACDF59508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{018EB189-D9A7-46AA-BE2A-B3BAA71C270A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="E-Cooking" sheetId="1" r:id="rId1"/>
+    <sheet name="Electricity" sheetId="1" r:id="rId1"/>
     <sheet name="LPG" sheetId="2" r:id="rId2"/>
     <sheet name="Carbon" sheetId="3" r:id="rId3"/>
   </sheets>

</xml_diff>